<commit_message>
📊 Auto scan: 2026-04-26
</commit_message>
<xml_diff>
--- a/archive/2026-04-26/report.xlsx
+++ b/archive/2026-04-26/report.xlsx
@@ -566,7 +566,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -576,7 +576,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -603,7 +603,7 @@
   <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -664,7 +664,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>페이커</t>
+          <t>첼시 대 리즈 유나이티드</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -695,7 +695,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>kacey musgraves</t>
+          <t>arsenal vs lyon</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -747,7 +747,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Ape Wisdom | Trending Stocks on Reddit</t>
+          <t>Ape Wisdom | Trending Stocks on r/wallstreetbets</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -757,43 +757,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>deion sanders</t>
+          <t>관련주</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>2</v>
-      </c>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
-        <v>96</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>박현경</t>
+          <t>테마주</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -801,57 +801,61 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="n">
-        <v>96</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
+        <v>100</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2차전지</t>
+          <t>jessica pegula</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
       <c r="E7" t="n">
-        <v>95</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
-        <v>3.19</v>
-      </c>
+        <v>96</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>테마주</t>
+          <t>엘니뇨</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -859,30 +863,30 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
       <c r="E8" t="n">
-        <v>94</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>96</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
-        </is>
-      </c>
-      <c r="I8" t="n">
-        <v>8</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>수혜주</t>
+          <t>2차전지</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -892,23 +896,19 @@
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="n">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
-        </is>
-      </c>
-      <c r="I9" t="n">
-        <v>8</v>
-      </c>
+      <c r="G9" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>관련주</t>
+          <t>수혜주</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -929,7 +929,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
+          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -939,7 +939,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>gervonta davis</t>
+          <t>stuttgart fc</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -970,7 +970,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>김원훈</t>
+          <t>옥택연 결혼</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1001,7 +1001,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>bill perkins</t>
+          <t>ipl standings</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1032,7 +1032,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>파면</t>
+          <t>채무</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1063,7 +1063,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>김윤식</t>
+          <t>이동국</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1094,7 +1094,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>maitland ward</t>
+          <t>kkr vs lsg</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1125,7 +1125,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>genoa - como</t>
+          <t>real oviedo vs elche</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1156,7 +1156,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>김승현</t>
+          <t>크리스티아누 호날두</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1187,7 +1187,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Thematic</t>
+          <t>ETFs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1218,7 +1218,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ETFs</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1228,7 +1228,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
@@ -1239,7 +1239,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Thematic ETFs &amp;amp; thematic investing ideas | BlackRock</t>
+          <t>최근 주목받는 테마주 총정리! 2025년 투자자가 꼭 봐야 할 테마주도주 Top 10 : 네이버 블로그</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1249,38 +1249,38 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>jamie raskin</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>7</v>
+      </c>
       <c r="E21" t="n">
-        <v>78</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
+        <v>76</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>최근 주목받는 테마주 총정리! 2025년 투자자가 꼭 봐야 할 테마주도주 Top 10 : 네이버 블로그</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>6</v>
-      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>lorient vs strasbourg</t>
+          <t>오너</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1290,7 +1290,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1311,12 +1311,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>제시카</t>
+          <t>이차전지</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1324,45 +1324,45 @@
           <t>KR</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>7</v>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="n">
-        <v>76</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>73</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>2.45</v>
+      </c>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>이차전지</t>
+          <t>paul seixas</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>google</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>KR</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr"/>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>8</v>
+      </c>
       <c r="E24" t="n">
-        <v>73</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>2.45</v>
-      </c>
+        <v>72</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>RSS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
     </row>
@@ -1396,7 +1396,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>데이터 센터</t>
+          <t>담합</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1427,43 +1427,39 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>dino prizmic</t>
+          <t>캐즘</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>google</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>8</v>
-      </c>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
-        <v>72</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>RSS</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+        <v>71</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
+        <v>2.39</v>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>캐즘</t>
+          <t>총정리</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1473,19 +1469,23 @@
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>2.39</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>최근 주목받는 테마주 총정리! 2025년 투자자가 꼭 봐야 할 테마주도주 Top 10 : 네이버 블로그</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Thematic</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1506,7 +1506,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Top Trending WallStreetBets Stocks (WSB) in Last 24hrs - LIVE</t>
+          <t>Thematic ETFs &amp;amp; thematic investing ideas | BlackRock</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -1516,7 +1516,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>최정윤</t>
+          <t>박현경</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1547,7 +1547,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>jeopardy longest winning streaks</t>
+          <t>real oviedo - elche c. f.</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ej smith</t>
+          <t>stuttgart - werder bremen</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1636,7 +1636,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>두산</t>
+          <t>김원훈</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1667,7 +1667,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>총정리</t>
+          <t>네이버</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1688,7 +1688,7 @@
       <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
-          <t>테마별 대장주 총정리! 업종별 1등주만 모았다</t>
+          <t>최근 주목받는 테마주 총정리! 2025년 투자자가 꼭 봐야 할 테마주도주 Top 10 : 네이버 블로그</t>
         </is>
       </c>
       <c r="I35" t="n">
@@ -1698,7 +1698,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Reddit</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1719,7 +1719,7 @@
       <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
-          <t>wallstreetbets - Reddit</t>
+          <t>Top Trending WallStreetBets Stocks (WSB) in Last 24hrs - LIVE</t>
         </is>
       </c>
       <c r="I36" t="n">
@@ -1729,7 +1729,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>블로그</t>
+          <t>wallstreetbets</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
@@ -1750,7 +1750,7 @@
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
-          <t>최근 주목받는 테마주 총정리! 2025년 투자자가 꼭 봐야 할 테마주도주 Top 10 : 네이버 블로그</t>
+          <t>wallstreetbets - Reddit</t>
         </is>
       </c>
       <c r="I37" t="n">
@@ -1787,7 +1787,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Today</t>
+          <t>WallStreetBets</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1808,7 +1808,7 @@
       <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Most Mentioned Reddit Stocks Today | WallStreetBets Top 100</t>
+          <t>Top Trending WallStreetBets Stocks (WSB) in Last 24hrs - LIVE</t>
         </is>
       </c>
       <c r="I39" t="n">
@@ -1818,7 +1818,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>네이버</t>
+          <t>블로그</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1849,65 +1849,65 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ETF</t>
+          <t>전고체</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Thematic ETF-Of-ETFs Launches - ETF.com</t>
-        </is>
-      </c>
-      <c r="I41" t="n">
-        <v>4</v>
-      </c>
+      <c r="G41" t="n">
+        <v>1.97</v>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>전고체</t>
+          <t>Trending</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="n">
-        <v>1.97</v>
-      </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="I42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Ape Wisdom | Trending Stocks on r/wallstreetbets</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>이재명</t>
+          <t>Reddit</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1928,7 +1928,7 @@
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
-          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
+          <t>wallstreetbets - Reddit</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -1938,7 +1938,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Trending</t>
+          <t>com</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1948,7 +1948,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1959,7 +1959,7 @@
       <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Ape Wisdom | Trending Stocks on Reddit</t>
+          <t>코스피 (KS11) - Investing.com</t>
         </is>
       </c>
       <c r="I44" t="n">
@@ -1969,7 +1969,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>실시간</t>
+          <t>코스피</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
-          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
+          <t>코스피 (KS11) - Investing.com</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -2000,7 +2000,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>com</t>
+          <t>실시간</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2021,7 +2021,7 @@
       <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
-          <t>코스피 (KS11) - Investing.com</t>
+          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -2031,7 +2031,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>amp</t>
+          <t>Best</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2052,7 +2052,7 @@
       <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Stock Market Movers Today • Top Gainers &amp;amp; Losers - Benzinga</t>
+          <t>This Week&amp;#x27;s Best Performing Stocks, Sectors, Industries Rankings ...</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -2062,7 +2062,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>com</t>
+          <t>amp</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2083,7 +2083,7 @@
       <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Top 100 most popular meme stocks today - feargreedmeter.com</t>
+          <t>Sector &amp;amp; Industry Performance - Bloomberg</t>
         </is>
       </c>
       <c r="I48" t="n">
@@ -2093,7 +2093,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>WallStreetBets</t>
+          <t>Most</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2114,7 +2114,7 @@
       <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Top Trending WallStreetBets Stocks (WSB) in Last 24hrs - LIVE</t>
+          <t>Reddit Wallstreetbets - Most Active Stocks - Tradestie</t>
         </is>
       </c>
       <c r="I49" t="n">
@@ -2124,7 +2124,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Most</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2155,7 +2155,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Buy</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2176,7 +2176,7 @@
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Reddit Wallstreetbets - Most Active Stocks - Tradestie</t>
+          <t>Hot Stocks to Buy for Today &amp;amp; Tomorrow | InvestorPlace</t>
         </is>
       </c>
       <c r="I51" t="n">
@@ -2186,7 +2186,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>대장주</t>
+          <t>이재명</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2207,7 +2207,7 @@
       <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
-          <t>테마별 대장주 총정리! 업종별 1등주만 모았다</t>
+          <t>이재명 관련주 - 정책 수혜주 Top 10 총정리 (2025 최신판)</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -2217,38 +2217,34 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>원전 수출</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>naver</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Today&amp;#x27;s Most Active Stocks - Stock Analysis</t>
-        </is>
-      </c>
-      <c r="I53" t="n">
-        <v>3</v>
-      </c>
+      <c r="G53" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>원전 수출</t>
+          <t>신한울</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2263,11 +2259,11 @@
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
-        <v>1.78</v>
+        <v>1.72</v>
       </c>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
@@ -2275,7 +2271,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>신한울</t>
+          <t>하이브</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2290,11 +2286,11 @@
       </c>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>1.72</v>
+        <v>1.67</v>
       </c>
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr"/>
@@ -2302,7 +2298,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>하이브</t>
+          <t>엔드포인트</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2356,7 +2352,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>엔드포인트</t>
+          <t>배터리 셀</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2371,11 +2367,11 @@
       </c>
       <c r="D58" t="inlineStr"/>
       <c r="E58" t="n">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="n">
-        <v>1.67</v>
+        <v>1.64</v>
       </c>
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr"/>
@@ -2383,7 +2379,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>배터리 셀</t>
+          <t>르세라핌</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2398,11 +2394,11 @@
       </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="n">
-        <v>1.64</v>
+        <v>1.57</v>
       </c>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
@@ -2410,7 +2406,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>르세라핌</t>
+          <t>그린수소</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2429,7 +2425,7 @@
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="n">
-        <v>1.57</v>
+        <v>1.59</v>
       </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
@@ -2437,12 +2433,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>그린수소</t>
+          <t>급상승</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>naver</t>
+          <t>web</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2452,14 +2448,18 @@
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F61" t="inlineStr"/>
-      <c r="G61" t="n">
-        <v>1.59</v>
-      </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>실시간 테마주 순위 | 급상승 테마 관련주 정보 - 알파스퀘어</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -13157,7 +13157,7 @@
     <col width="14" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -13638,7 +13638,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>70.09999999999999</v>
+        <v>74.3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -13649,7 +13649,7 @@
         <v>68.90000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>68.8</v>
+        <v>80.7</v>
       </c>
       <c r="J9" t="n">
         <v>75</v>
@@ -13659,12 +13659,12 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2차전지, 이차전지, 캐즘, 양극재, 전고체</t>
+          <t>jessica pegula, 2차전지, 이차전지, 캐즘, 양극재</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 69점 (2주avg/4-8주avg = 2.56, 2주/2-4주 = 2.45). 트렌드 시그널 69점 — 매칭 키워드: 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점), 전고체(naver, 59점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: CNT 도전재</t>
+          <t>[테마: 2차전지/배터리] 거래량 시그널 69점 (2주avg/4-8주avg = 2.56, 2주/2-4주 = 2.45). 트렌드 시그널 81점 — 매칭 키워드: jessica pegula(google, 96점), 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: CNT 도전재</t>
         </is>
       </c>
     </row>
@@ -13693,7 +13693,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>61.2</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -13704,7 +13704,7 @@
         <v>49.2</v>
       </c>
       <c r="I10" t="n">
-        <v>68.8</v>
+        <v>80.7</v>
       </c>
       <c r="J10" t="n">
         <v>75</v>
@@ -13714,24 +13714,24 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2차전지, 이차전지, 캐즘, 양극재, 전고체</t>
+          <t>jessica pegula, 2차전지, 이차전지, 캐즘, 양극재</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 49점 (2주avg/4-8주avg = 1.64, 2주/2-4주 = 1.11). 트렌드 시그널 69점 — 매칭 키워드: 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점), 전고체(naver, 59점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: 프리미엄 셀</t>
+          <t>[테마: 2차전지/배터리] 거래량 시그널 49점 (2주avg/4-8주avg = 1.64, 2주/2-4주 = 1.11). 트렌드 시그널 81점 — 매칭 키워드: jessica pegula(google, 96점), 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: 프리미엄 셀</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>000990</t>
+          <t>373220</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -13740,53 +13740,53 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>152000</v>
+        <v>481000</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AI/반도체</t>
+          <t>2차전지/배터리</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>59.5</v>
+        <v>62.6</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>⚪ 관찰</t>
+          <t>🟡 주목</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>58</v>
+        <v>43.1</v>
       </c>
       <c r="I11" t="n">
-        <v>81</v>
+        <v>80.7</v>
       </c>
       <c r="J11" t="n">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>maitland ward, HBM3</t>
+          <t>jessica pegula, 2차전지, 이차전지, 캐즘, 양극재</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>[테마: AI/반도체] 거래량 시그널 58점 (2주avg/4-8주avg = 1.93, 2주/2-4주 = 1.71). 트렌드 시그널 81점 — 매칭 키워드: maitland ward(google, 84점), HBM3(naver, 62점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 특화 파운드리</t>
+          <t>[테마: 2차전지/배터리] 거래량 시그널 43점 (2주avg/4-8주avg = 1.44, 2주/2-4주 = 1.12). 트렌드 시그널 81점 — 매칭 키워드: jessica pegula(google, 96점), 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: 글로벌 2위 셀</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>373220</t>
+          <t>000990</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -13795,15 +13795,15 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>481000</v>
+        <v>152000</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2차전지/배터리</t>
+          <t>AI/반도체</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>58.5</v>
+        <v>52.8</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -13811,25 +13811,25 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>43.1</v>
+        <v>58</v>
       </c>
       <c r="I12" t="n">
-        <v>68.8</v>
+        <v>62</v>
       </c>
       <c r="J12" t="n">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2차전지, 이차전지, 캐즘, 양극재, 전고체</t>
+          <t>HBM3</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>[테마: 2차전지/배터리] 거래량 시그널 43점 (2주avg/4-8주avg = 1.44, 2주/2-4주 = 1.12). 트렌드 시그널 69점 — 매칭 키워드: 2차전지(naver, 95점), 이차전지(naver, 73점), 캐즘(naver, 71점), 양극재(naver, 66점), 전고체(naver, 59점). 동일 테마 동시통과 3종목(밀집도 75점). 종목 근거: 글로벌 2위 셀</t>
+          <t>[테마: AI/반도체] 거래량 시그널 58점 (2주avg/4-8주avg = 1.93, 2주/2-4주 = 1.71). 트렌드 시그널 62점 — 매칭 키워드: HBM3(naver, 62점). 동일 테마 동시통과 1종목(밀집도 25점). 종목 근거: 특화 파운드리</t>
         </is>
       </c>
     </row>

</xml_diff>